<commit_message>
Fix up double institutes:
</commit_message>
<xml_diff>
--- a/11-CollaborationList/Imperial.xlsx
+++ b/11-CollaborationList/Imperial.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://api.box.com/wopi/files/2050113224685/WOPIServiceId_TP_BOX_2/WOPIUserId_-/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{96E5052D-56CD-784F-9B91-457CD138E2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7878E71E-2A78-9D49-9A12-EA3B692F8344}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{96E5052D-56CD-784F-9B91-457CD138E2B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A559A5BC-4A3E-934C-A6E8-6B86D497F2BE}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{7B5F04B9-63DF-474E-BF2F-8D8D82A0D772}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="186">
   <si>
     <t>Title</t>
   </si>
@@ -236,12 +236,6 @@
   </si>
   <si>
     <t>Josie M. McGarrigle </t>
-  </si>
-  <si>
-    <t>Inst-Curie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Institut Curie,  73 Rue Claude Bernard,  75005, Paris, France </t>
   </si>
   <si>
     <t>Roland</t>
@@ -1556,28 +1550,28 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C2" t="s">
         <v>154</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>155</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D2" t="s">
+      <c r="F2" t="s">
         <v>157</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="F2" t="s">
-        <v>159</v>
-      </c>
       <c r="G2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="H2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -1585,28 +1579,28 @@
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D3" t="s">
         <v>141</v>
       </c>
-      <c r="B3" t="s">
+      <c r="E3" s="1" t="s">
         <v>142</v>
       </c>
-      <c r="C3" t="s">
-        <v>169</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>143</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="G3" t="s">
         <v>144</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>145</v>
-      </c>
-      <c r="G3" t="s">
-        <v>146</v>
-      </c>
-      <c r="H3" t="s">
-        <v>147</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -1635,7 +1629,7 @@
         <v>22</v>
       </c>
       <c r="H4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -1667,7 +1661,7 @@
         <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="I5">
         <v>0</v>
@@ -1699,7 +1693,7 @@
         <v>38</v>
       </c>
       <c r="H6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1731,7 +1725,7 @@
         <v>44</v>
       </c>
       <c r="H7" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -1763,7 +1757,7 @@
         <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -1815,37 +1809,37 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B10" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" t="s">
         <v>160</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
+        <v>161</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10" t="s">
         <v>162</v>
-      </c>
-      <c r="D10" t="s">
-        <v>163</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="F10" t="s">
-        <v>164</v>
       </c>
       <c r="G10" t="s">
         <v>64</v>
       </c>
       <c r="H10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I10">
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K10" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
@@ -1853,69 +1847,69 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C11" t="s">
+        <v>102</v>
+      </c>
+      <c r="D11" t="s">
         <v>103</v>
       </c>
-      <c r="C11" t="s">
+      <c r="E11" t="s">
         <v>104</v>
       </c>
-      <c r="D11" t="s">
+      <c r="F11" t="s">
         <v>105</v>
-      </c>
-      <c r="E11" t="s">
-        <v>106</v>
-      </c>
-      <c r="F11" t="s">
-        <v>107</v>
       </c>
       <c r="G11" t="s">
         <v>64</v>
       </c>
       <c r="H11" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I11">
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K11" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" t="s">
         <v>149</v>
-      </c>
-      <c r="B12" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" t="s">
-        <v>151</v>
       </c>
       <c r="D12" t="s">
         <v>50</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G12" t="s">
         <v>64</v>
       </c>
       <c r="H12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I12">
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
@@ -1941,7 +1935,7 @@
         <v>64</v>
       </c>
       <c r="H13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I13">
         <v>1</v>
@@ -1950,7 +1944,7 @@
         <v>38</v>
       </c>
       <c r="K13" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="N13" t="s">
         <v>65</v>
@@ -1964,40 +1958,40 @@
         <v>16</v>
       </c>
       <c r="B14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C14" t="s">
+        <v>175</v>
+      </c>
+      <c r="D14" t="s">
         <v>176</v>
       </c>
-      <c r="C14" t="s">
+      <c r="E14" t="s">
         <v>177</v>
       </c>
-      <c r="D14" t="s">
+      <c r="F14" t="s">
         <v>178</v>
-      </c>
-      <c r="E14" t="s">
-        <v>179</v>
-      </c>
-      <c r="F14" t="s">
-        <v>180</v>
       </c>
       <c r="G14" t="s">
         <v>64</v>
       </c>
       <c r="H14" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I14">
         <v>1</v>
       </c>
       <c r="J14" t="s">
+        <v>82</v>
+      </c>
+      <c r="K14" t="s">
+        <v>83</v>
+      </c>
+      <c r="L14" t="s">
         <v>84</v>
       </c>
-      <c r="K14" t="s">
-        <v>85</v>
-      </c>
-      <c r="L14" t="s">
-        <v>86</v>
-      </c>
       <c r="M14" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -2005,40 +1999,40 @@
         <v>32</v>
       </c>
       <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" t="s">
+        <v>78</v>
+      </c>
+      <c r="D15" t="s">
         <v>79</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E15" t="s">
         <v>80</v>
       </c>
-      <c r="D15" t="s">
+      <c r="F15" t="s">
         <v>81</v>
-      </c>
-      <c r="E15" t="s">
-        <v>82</v>
-      </c>
-      <c r="F15" t="s">
-        <v>83</v>
       </c>
       <c r="G15" t="s">
         <v>64</v>
       </c>
       <c r="H15" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I15">
         <v>2</v>
       </c>
       <c r="J15" t="s">
+        <v>82</v>
+      </c>
+      <c r="K15" t="s">
+        <v>83</v>
+      </c>
+      <c r="L15" t="s">
         <v>84</v>
       </c>
-      <c r="K15" t="s">
-        <v>85</v>
-      </c>
-      <c r="L15" t="s">
-        <v>86</v>
-      </c>
       <c r="M15" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -2046,34 +2040,34 @@
         <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="G16" t="s">
         <v>64</v>
       </c>
       <c r="H16" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I16">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K16" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
@@ -2081,43 +2075,43 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
+        <v>106</v>
+      </c>
+      <c r="C17" t="s">
+        <v>107</v>
+      </c>
+      <c r="D17" t="s">
         <v>108</v>
       </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
+        <v>146</v>
+      </c>
+      <c r="F17" t="s">
         <v>109</v>
-      </c>
-      <c r="D17" t="s">
-        <v>110</v>
-      </c>
-      <c r="E17" t="s">
-        <v>148</v>
-      </c>
-      <c r="F17" t="s">
-        <v>111</v>
       </c>
       <c r="G17" t="s">
         <v>64</v>
       </c>
       <c r="H17" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I17">
         <v>2</v>
       </c>
       <c r="J17" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L17" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="M17" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
@@ -2125,43 +2119,43 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" t="s">
         <v>91</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" t="s">
         <v>92</v>
       </c>
-      <c r="D18" t="s">
-        <v>93</v>
-      </c>
-      <c r="E18" t="s">
-        <v>94</v>
-      </c>
       <c r="F18" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G18" t="s">
         <v>64</v>
       </c>
       <c r="H18" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I18">
         <v>2</v>
       </c>
       <c r="J18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L18" t="s">
+        <v>93</v>
+      </c>
+      <c r="M18" t="s">
+        <v>94</v>
+      </c>
+      <c r="N18" t="s">
         <v>95</v>
-      </c>
-      <c r="M18" t="s">
-        <v>96</v>
-      </c>
-      <c r="N18" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
@@ -2187,16 +2181,10 @@
         <v>64</v>
       </c>
       <c r="H19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I19">
-        <v>1</v>
-      </c>
-      <c r="J19" t="s">
-        <v>72</v>
-      </c>
-      <c r="K19" t="s">
-        <v>73</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
@@ -2204,37 +2192,37 @@
         <v>24</v>
       </c>
       <c r="B20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" t="s">
+        <v>112</v>
+      </c>
+      <c r="D20" t="s">
         <v>113</v>
       </c>
-      <c r="C20" t="s">
+      <c r="E20" t="s">
         <v>114</v>
       </c>
-      <c r="D20" t="s">
+      <c r="F20" t="s">
         <v>115</v>
-      </c>
-      <c r="E20" t="s">
-        <v>116</v>
-      </c>
-      <c r="F20" t="s">
-        <v>117</v>
       </c>
       <c r="G20" t="s">
         <v>64</v>
       </c>
       <c r="H20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I20">
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K20" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="N20" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.2">
@@ -2242,40 +2230,40 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" t="s">
+        <v>97</v>
+      </c>
+      <c r="D21" t="s">
         <v>98</v>
       </c>
-      <c r="C21" t="s">
+      <c r="E21" t="s">
         <v>99</v>
       </c>
-      <c r="D21" t="s">
+      <c r="F21" t="s">
         <v>100</v>
-      </c>
-      <c r="E21" t="s">
-        <v>101</v>
-      </c>
-      <c r="F21" t="s">
-        <v>102</v>
       </c>
       <c r="G21" t="s">
         <v>64</v>
       </c>
       <c r="H21" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I21">
         <v>2</v>
       </c>
       <c r="J21" t="s">
+        <v>82</v>
+      </c>
+      <c r="K21" t="s">
+        <v>83</v>
+      </c>
+      <c r="L21" t="s">
         <v>84</v>
       </c>
-      <c r="K21" t="s">
-        <v>85</v>
-      </c>
-      <c r="L21" t="s">
-        <v>86</v>
-      </c>
       <c r="M21" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.2">
@@ -2283,60 +2271,60 @@
         <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C22" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D22" t="s">
         <v>41</v>
       </c>
       <c r="E22" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F22" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G22" t="s">
         <v>64</v>
       </c>
       <c r="H22" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I22">
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="K22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B23" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C23" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D23" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F23" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G23" t="s">
         <v>64</v>
       </c>
       <c r="H23" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -2347,25 +2335,25 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" t="s">
+        <v>73</v>
+      </c>
+      <c r="D24" t="s">
         <v>74</v>
       </c>
-      <c r="C24" t="s">
+      <c r="E24" t="s">
         <v>75</v>
       </c>
-      <c r="D24" t="s">
+      <c r="F24" t="s">
         <v>76</v>
-      </c>
-      <c r="E24" t="s">
-        <v>77</v>
-      </c>
-      <c r="F24" t="s">
-        <v>78</v>
       </c>
       <c r="G24" t="s">
         <v>64</v>
       </c>
       <c r="H24" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I24">
         <v>0</v>
@@ -2373,28 +2361,28 @@
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B25" t="s">
+        <v>169</v>
+      </c>
+      <c r="C25" t="s">
+        <v>170</v>
+      </c>
+      <c r="D25" t="s">
+        <v>183</v>
+      </c>
+      <c r="E25" t="s">
+        <v>173</v>
+      </c>
+      <c r="F25" t="s">
         <v>171</v>
-      </c>
-      <c r="C25" t="s">
-        <v>172</v>
-      </c>
-      <c r="D25" t="s">
-        <v>185</v>
-      </c>
-      <c r="E25" t="s">
-        <v>175</v>
-      </c>
-      <c r="F25" t="s">
-        <v>173</v>
       </c>
       <c r="G25" t="s">
         <v>64</v>
       </c>
       <c r="H25" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I25">
         <v>0</v>
@@ -2402,28 +2390,28 @@
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
+        <v>163</v>
+      </c>
+      <c r="C26" t="s">
+        <v>166</v>
+      </c>
+      <c r="D26" t="s">
+        <v>182</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="F26" t="s">
         <v>165</v>
       </c>
-      <c r="C26" t="s">
-        <v>168</v>
-      </c>
-      <c r="D26" t="s">
-        <v>184</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="F26" t="s">
-        <v>167</v>
-      </c>
       <c r="G26" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H26" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I26">
         <v>0</v>
@@ -2434,25 +2422,25 @@
         <v>24</v>
       </c>
       <c r="B27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C27" t="s">
+        <v>124</v>
+      </c>
+      <c r="D27" t="s">
         <v>125</v>
       </c>
-      <c r="C27" t="s">
+      <c r="E27" t="s">
         <v>126</v>
       </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
         <v>127</v>
       </c>
-      <c r="E27" t="s">
-        <v>128</v>
-      </c>
-      <c r="F27" t="s">
-        <v>129</v>
-      </c>
       <c r="G27" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H27" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I27">
         <v>0</v>
@@ -2466,31 +2454,31 @@
         <v>24</v>
       </c>
       <c r="B28" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" t="s">
         <v>119</v>
       </c>
-      <c r="C28" t="s">
+      <c r="E28" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" t="s">
         <v>120</v>
       </c>
-      <c r="D28" t="s">
+      <c r="G28" t="s">
         <v>121</v>
       </c>
-      <c r="E28" t="s">
-        <v>140</v>
-      </c>
-      <c r="F28" t="s">
-        <v>122</v>
-      </c>
-      <c r="G28" t="s">
-        <v>123</v>
-      </c>
       <c r="H28" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I28">
         <v>0</v>
       </c>
       <c r="O28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>